<commit_message>
fix: seperate astri and stella
</commit_message>
<xml_diff>
--- a/magik/rwi_stela_integration/resources/template HPDB astri.xlsx
+++ b/magik/rwi_stela_integration/resources/template HPDB astri.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12300"/>
+    <workbookView windowWidth="12285" windowHeight="4485" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="CLUSTER" sheetId="1" r:id="rId1"/>
@@ -1366,7 +1366,7 @@
     <col min="11" max="11" width="15.1428571428571" customWidth="1"/>
     <col min="12" max="12" width="11.7142857142857" customWidth="1"/>
     <col min="13" max="13" width="14.1428571428571" customWidth="1"/>
-    <col min="14" max="14" width="12.5714285714286" customWidth="1"/>
+    <col min="14" max="14" width="14.7142857142857" customWidth="1"/>
     <col min="15" max="15" width="12" customWidth="1"/>
     <col min="16" max="16" width="43.2857142857143" customWidth="1"/>
     <col min="17" max="17" width="13.7142857142857" customWidth="1"/>
@@ -2967,7 +2967,7 @@
       <c r="U2"/>
       <c r="V2" s="12"/>
       <c r="AB2" s="12"/>
-      <c r="AC2"/>
+      <c r="AC2" s="10"/>
       <c r="AD2" s="11"/>
       <c r="AE2" s="10"/>
       <c r="AF2"/>
@@ -3003,7 +3003,7 @@
       <c r="U3"/>
       <c r="V3" s="12"/>
       <c r="AB3" s="12"/>
-      <c r="AC3"/>
+      <c r="AC3" s="10"/>
       <c r="AD3" s="11"/>
       <c r="AE3" s="10"/>
       <c r="AF3"/>

</xml_diff>